<commit_message>
Add admin impact workflow and mobile polish
</commit_message>
<xml_diff>
--- a/tasks/tenant-graph-feature-stories.xlsx
+++ b/tasks/tenant-graph-feature-stories.xlsx
@@ -1,26 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="Feature Stories" sheetId="1" r:id="rId1"/>
-    <sheet name="Test Runs" sheetId="2" r:id="rId2"/>
-    <sheet name="Errors" sheetId="3" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Stories" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
+      <name val="Aptos"/>
       <sz val="11"/>
-      <name val="Aptos"/>
     </font>
   </fonts>
   <fills count="1">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
   </fills>
   <borders count="1">
@@ -36,33 +39,388 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N89"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N96"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="42" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
-    <col min="6" max="6" width="42" customWidth="1"/>
-    <col min="7" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="22" customWidth="1"/>
-    <col min="10" max="10" width="42" customWidth="1"/>
-    <col min="11" max="11" width="42" customWidth="1"/>
-    <col min="12" max="12" width="22" customWidth="1"/>
-    <col min="13" max="13" width="42" customWidth="1"/>
-    <col min="14" max="14" width="42" customWidth="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -188,19 +546,9 @@
           <t>Missing config behavior is covered by missingRequiredEnvVars unit test and App source rendering MissingConfigScreen when hasMsalConfig is false.</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -260,19 +608,9 @@
           <t>Browser/live tenant pass. localhost redirect normalized; popup returned to app workspace instead of nested prompt.</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -332,19 +670,9 @@
           <t>Browser/live tenant pass. Clicked Sign In in stale anonymous tab; MSAL popup opened and completed to authenticated workspace.</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -476,19 +804,9 @@
           <t>Browser/live tenant pass. Authenticated workspace shows active Break Glass account.</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -548,19 +866,9 @@
           <t>Browser/live tenant pass. Live Graph calls loaded tenant overview and sign-in logs.</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -620,19 +928,9 @@
           <t>Live sign-out clicked account menu, redirected to Microsoft account picker, selected account, and returned Tenant Graph to its sign-in screen. Re-auth popup opened afterward.</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -692,19 +990,9 @@
           <t>Account menu external links were intercepted with window.open: Profile opens myaccount.microsoft.com and Tenant switch opens /organizations.</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -764,19 +1052,9 @@
           <t>Browser/live tenant pass. Sign-in screen retains Vanta NET background; previous smoke plus anonymous tab confirmed prompt.</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -836,19 +1114,9 @@
           <t>Browser/live tenant pass. Live tenant overview loaded 176 objects and 96 relationships.</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -908,19 +1176,9 @@
           <t>Automated collectGraphs test verifies fulfilled graph data is preserved while warning and permission errors are aggregated.</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -980,19 +1238,9 @@
           <t>Browser/live tenant pass. Reset flow showed loading while tenant graph reloaded.</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1052,19 +1300,9 @@
           <t>Browser/live tenant pass. Disabling object types produced 0 objects, 0 relationships, and explicit no-visible-objects copy.</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1124,19 +1362,9 @@
           <t>Browser/live tenant pass. Reset returned to 176 objects / 96 relationships after projected sign-in state.</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1196,19 +1424,9 @@
           <t>Browser/live tenant pass. Toolbar search for iOS returned five relevant Intune objects.</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1340,19 +1558,9 @@
           <t>Automated unit/type/build evidence. Unit coverage verifies local fallback/no-query result behavior.</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1412,19 +1620,9 @@
           <t>Browser/live tenant pass. Top iOS results were exact/prefix matches before broader matches.</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1484,19 +1682,9 @@
           <t>Browser/live tenant pass. Load 30 more increased result rows from 30 to 60.</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1628,19 +1816,9 @@
           <t>Relationship type filter verified live: disabling Scope tag reduced visible relationships from 96 to 2 and restoring the checkbox restored the relationship set.</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1700,19 +1878,9 @@
           <t>Browser/live tenant pass. Default graph cap is active; overview remains bounded and paged.</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1772,19 +1940,9 @@
           <t>Three.js scene lifecycle is covered by source cleanup inspection and sign-out/unmount browser evidence: app returns to sign-in screen with no graph canvas. Cleanup removes listeners, controls, disposed objects, renderer, and canvas.</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -1844,19 +2002,9 @@
           <t>Browser/live tenant pass. Desktop screenshot shows typed icons and OS/type legend.</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -1926,11 +2074,6 @@
           <t>No fix needed</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="N26" t="inlineStr">
         <is>
           <t>Expected missing profile-photo 404 does not block graph load and falls back to glyph.</t>
@@ -1988,19 +2131,9 @@
           <t>Browser/live tenant pass. Desktop screenshot shows semantic cluster zones and labels.</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2060,19 +2193,9 @@
           <t>Browser/live tenant pass. Selected Break Glass node renders with dominant halo and label.</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2132,19 +2255,9 @@
           <t>Relationship visual policy tests cover assignment, membership dashed, primary-user double-line, filtered-by dotted, detected-app animated, scope-tag thin styles, and direction endpoints.</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2204,19 +2317,9 @@
           <t>Focus depth controls verified live: Direct value 1, Two-Hop value 2, and Off value 0 all apply and reset without breaking the graph.</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2276,19 +2379,9 @@
           <t>Zoom/pan/rotate gestures were exercised on the Three.js canvas, then Fit restored a usable graph viewport.</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2348,19 +2441,9 @@
           <t>Coordinate sweep found node tooltip for an assignment filter; tooltip showed label, type, relationship count, and metadata.</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2420,19 +2503,9 @@
           <t>Direct graph-node click verified from a tooltip-discovered canvas coordinate; clicked settings catalog policy pinned matching details.</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2492,19 +2565,9 @@
           <t>Canvas edge click selected a Scope tag relationship and opened the inspector breadcrumb/relationship detail.</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2564,19 +2627,9 @@
           <t>Canvas cluster click isolated policy object types and zoomed to 113 policy objects / 0 relationships.</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2636,19 +2689,9 @@
           <t>Browser/live tenant pass. Fit and View controls stayed clickable and preserved canvas.</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2708,19 +2751,9 @@
           <t>Progressive label priority and collision behavior are covered by graphVisualPolicy label-priority tests, graphLabelVisibility collision tests, and live screenshots/label visibility evidence.</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2780,19 +2813,9 @@
           <t>Browser/live tenant pass. Legend visible with Windows, iOS, Users, Roles, Apps, Policies, Filters, Scope tags, Groups.</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L38" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2852,19 +2875,9 @@
           <t>Browser/live tenant pass. Mini map visible with selected marker and count.</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L39" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2924,19 +2937,9 @@
           <t>No-selection state is covered by DetailsPanel server-render test, which verifies the Selection panel renders Select an object to explain it when no node is selected.</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L40" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2996,19 +2999,9 @@
           <t>Browser/live tenant pass. Selected object details panel and inspector show Break Glass metadata.</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L41" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3068,19 +3061,9 @@
           <t>Browser/live tenant pass. Expanded/no-expansion states are visible and disabled when no action is available.</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L42" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3140,19 +3123,9 @@
           <t>Browser/live tenant pass. Friendly summaries visible for user, assignment filter, and sign-in event objects.</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L43" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3212,19 +3185,9 @@
           <t>Friendly Names technical-details disclosure opened from collapsed state and showed Type/upn metadata, then closed cleanly.</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L44" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3284,19 +3247,9 @@
           <t>Browser/live tenant pass. At-a-glance cluster summary visible and readable.</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L45" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3356,19 +3309,9 @@
           <t>Data confidence signals are driven by permissionError/warnings; collectGraphs test verifies permissionError propagation and Sidebar source renders Missing permission/Partial data badges.</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L46" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3428,19 +3371,9 @@
           <t>Readable path finder positive path is covered by existing explainReadablePath/readablePathCandidates tests, and live UI showed explicit partial-data state.</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L47" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3500,19 +3433,9 @@
           <t>Admin mode renders Evidence drawer with normalized, metadata, and raw Graph fields for the selected object.</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L48" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3572,19 +3495,9 @@
           <t>Browser/live tenant pass. Right-side inspector is visible and close/copy controls are exposed.</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L49" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3644,19 +3557,9 @@
           <t>Edge click opened the relationship inspector with breadcrumb source, relationship label, and target object copy.</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L50" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3716,19 +3619,9 @@
           <t>Browser/live tenant pass. Copy name action clicked without page error; copy/link buttons visible.</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L51" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3788,19 +3681,9 @@
           <t>Intune and Entra inspector buttons were intercepted with window.open and produced admin-center URLs.</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L52" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3860,19 +3743,9 @@
           <t>Browser/live tenant pass. Relationships, assignments, filters, scope tags, and sign-ins sections render in inspector.</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L53" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3932,19 +3805,9 @@
           <t>Relationship inspector exposes Raw Graph IDs, Copy ID, and Graph query actions for the selected object.</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -4004,19 +3867,9 @@
           <t>Browser/live tenant pass. Sign-ins panel appears for selected user.</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L55" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -4076,19 +3929,9 @@
           <t>Browser/live tenant pass. Range, CA, result filters and bounded load button are visible and functional.</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L56" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4148,19 +3991,9 @@
           <t>Browser/live tenant pass. CA details scope path returned report-only Conditional Access policy counts.</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4220,19 +4053,9 @@
           <t>Sign-in load-more adapter now has explicit nextLink coverage: loadSignInLogs uses the provided Microsoft Graph nextLink and returns the next page token.</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4292,19 +4115,9 @@
           <t>Browser/live tenant pass. Sign-in summary showed Success and Report-only impact counts.</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L59" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4364,19 +4177,9 @@
           <t>Browser/live tenant pass. Clicking a sign-in event opened detailed sign-in fields.</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L60" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4436,19 +4239,9 @@
           <t>Missing sign-in/CA permission copy is covered by a forced GraphError(403) regression test and source-rendered warning state.</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L61" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4508,19 +4301,9 @@
           <t>Browser/live tenant pass. Projecting a sign-in event increased graph objects from 177 to 180, then reset removed it.</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L62" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4580,19 +4363,9 @@
           <t>Automated unit/type/build evidence. Typecheck/tests verify normalized TenantGraph/TenantNode/TenantEdge contracts.</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L63" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4652,19 +4425,9 @@
           <t>Automated unit/type/build evidence. Adapter tests verify Graph response normalization paths.</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L64" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4724,19 +4487,9 @@
           <t>Automated unit/type/build evidence. Directory role hydration tests verify display names instead of GUID labels.</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L65" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M65" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4796,19 +4549,9 @@
           <t>Automated unit/type/build evidence. Mobile app query fallback tests verify safe collection queries.</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L66" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4868,19 +4611,9 @@
           <t>Automated unit/type/build evidence. Broad assignment virtual-target tests prevent invalid expansion warnings.</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L67" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4940,19 +4673,9 @@
           <t>Progressive expansion state verified on a settings catalog policy: selected policy showed disabled Expanded depth 1 with guidance to increase relationship depth.</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L68" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -5012,19 +4735,9 @@
           <t>Browser/live tenant pass. Live CA classifier surfaced report-only impact; unit coverage also exercises classifier states.</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L69" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -5084,19 +4797,9 @@
           <t>Permission banners and graph warnings are backed by collectGraphs warning/permissionError propagation and AppShell/Sidebar source rendering.</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L70" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -5156,19 +4859,9 @@
           <t>Browser/live tenant pass. Mobile smoke had no horizontal overflow; toolbar, graph, legend, minimap fit 390px width.</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L71" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -5228,19 +4921,9 @@
           <t>Keyboard tour verified: fresh Tab order starts at search, reaches toolbar controls/account/results, Enter submits search, Tab reaches a result, and Enter pins details.</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L72" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5300,19 +4983,9 @@
           <t>Browser/live tenant pass. Reduced-motion source scan confirms centralized prefers-reduced-motion fallback.</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="L73" t="inlineStr">
         <is>
           <t>No fix needed</t>
-        </is>
-      </c>
-      <c r="M73" t="inlineStr">
-        <is>
-          <t/>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5632,7 +5305,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>The sample Graph client implements overview, search, expansion, assignments, sign-in logs, user photos, and app icon routes for users, groups, directory roles, devices, apps, policies, filters, scope tags, and Conditional Access data.</t>
+          <t>The sample Graph client implements overview, search, expansion, assignments, sign-in logs, user photos, app icons, and enlarged sample routes across users, groups, roles, devices, apps, policies, filters, scope tags, and Conditional Access data. Sample mode renders 81 objects / 37 relationships in the current default view.</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -5652,12 +5325,12 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-06-23 17:51 UTC</t>
+          <t>2026-06-24 04:03 UTC</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Focused tests: sample client overview/search/expand/sign-ins pass; browser shows users, devices, policies, apps, roles, sign-ins, and CA data.</t>
+          <t>Focused tests and Playwright sample smoke pass; browser sample mode shows 81 objects / 37 relationships and exercises users, devices, apps, policies, guardrails, sign-ins, CA data, app icons, and admin impact flows.</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5677,7 +5350,7 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>Validated in TR-027 sample tenant browser pass plus focused tests.</t>
+          <t>Updated after sample tenant expansion on codex/admin-impact-workflows.</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5377,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Sample apps are real apps with distinct Graph-style largeIcon data: Intune Company Portal, Microsoft Edge, Microsoft Defender, Windows App Mobile, SAP Concur, and Microsoft Outlook. Policy/configuration names must not appear as app nodes.</t>
+          <t>Sample apps are real apps with distinct icon data: Intune Company Portal, Microsoft Edge, Microsoft Defender, Windows App Mobile, SAP Concur, Microsoft Outlook, Microsoft Teams, Microsoft OneDrive, Zoom Workplace, Adobe Acrobat Reader, ServiceNow Agent, Salesforce, Slack, Microsoft Power BI, Microsoft Planner, and Microsoft Loop. Policy/configuration names must not appear as app nodes.</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -5724,12 +5397,12 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-06-23 17:51 UTC</t>
+          <t>2026-06-24 04:03 UTC</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Focused tests and browser text verify real apps: Intune Company Portal, Microsoft Edge, Microsoft Defender, Windows App Mobile, SAP Concur, Microsoft Outlook; no policy-shaped app label.</t>
+          <t>Focused tests verify all real app labels, no policy-shaped app labels, and distinct image data URLs; generated SVG app tiles cover added real apps without fake product names.</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5749,7 +5422,7 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>Validated in TR-027 sample tenant browser pass plus focused tests.</t>
+          <t>Updated after sample app catalog expansion.</t>
         </is>
       </c>
     </row>
@@ -6470,6 +6143,440 @@
       <c r="N89" t="inlineStr">
         <is>
           <t>Validated in TR-027 sample tenant browser pass plus focused tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>TG-089</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Sample tenant</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Large realistic sample tenant</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>As an evaluator, I want the sample tenant to feel like a real tenant so I can judge the product without connecting my environment.</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Sample mode includes 19 users, 15 groups, 19 managed devices, 16 managed apps, directory roles, compliance/configuration/settings/enrollment policies, assignment filters, scope tags, detected apps, memberships, assignments, and Conditional Access sign-in events. The initial sample view renders 81 objects / 37 relationships.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>src/demo/sampleTenantData.ts; src/demo/sampleTenantClient.ts; src/demo/sampleTenantClient.test.ts</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Automated unit test and Playwright sample smoke</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>2026-06-24 04:03 UTC</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>npx vitest sample tests pass; Playwright sample route reports 81 objects / 37 relationships, 17 people, 19 devices, 16 apps, 18 policies, and 11 guardrails.</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>No fix needed</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>Current sample tenant has enough variety for apps, groups, devices, policies, filters, roles, and sign-in investigation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>TG-090</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Admin investigation</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Impact analyzer blast radius</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>As an Intune or Entra admin, I want a selected object blast-radius summary so I can understand what may be affected before making a change.</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>The sidebar shows Impact analyzer for a selected object and Tenant hygiene when no object is selected. It displays loaded counts for users, devices, groups, apps, policies, and filters derived from the graph neighborhood.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>src/utils/adminInsights.ts; src/components/details/AdminImpactPanel.tsx; src/components/layout/workspaceSelectors.ts</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Unit test and Playwright browser smoke</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>2026-06-24 04:03 UTC</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>adminInsights unit tests pass; Playwright confirms Impact analyzer and blast-radius counts render in sample mode and update for Intune Company Portal selection.</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>No fix needed</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>Counts are intentionally scoped to loaded graph data, not guessed tenant totals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>TG-091</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Admin investigation</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Risk and hygiene review signals</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>As an admin, I want obvious risky relationships surfaced so I can focus review time on broad or blocking changes.</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>The admin panel flags broad All users/All devices targets, required assignments, noncompliant devices, privileged role membership visibility, and unconnected apps/policies in the loaded graph with severity-coded findings.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>src/utils/adminInsights.ts; src/utils/adminInsights.test.ts; src/components/details/AdminImpactPanel.tsx</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Unit test and Playwright browser smoke</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>2026-06-24 04:03 UTC</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Unit tests cover broad target, required assignment, noncompliant device, and selected-object findings; Playwright shows Company Portal review signals for required broad target assignment.</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>No fix needed</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>Findings are static rows, not dead clickable controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>TG-092</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Admin investigation</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Recent change investigation hints</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>As an admin troubleshooting a change, I want recently changed related policies called out so I know where to inspect audit logs.</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Nodes with recent created or modified metadata generate Recent changes entries that name the object, state whether it was created or modified, and advise checking audit logs before editing related assignments.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>src/utils/adminInsights.ts; src/components/details/AdminImpactPanel.tsx</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Unit test</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>2026-06-24 04:03 UTC</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>adminInsights unit test creates a recently modified settings catalog policy and verifies Recent changes output.</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>No fix needed</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>Uses loaded Graph metadata only; live audit-log correlation remains a future extension.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>TG-093</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Admin investigation</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Copyable investigation evidence</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>As an admin, I want one-click evidence text so I can paste the investigation into a ticket or change record.</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Copy evidence writes a concise text summary containing the selected subject, relationship count, blast radius, review findings, and recent change signals to the clipboard.</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>src/utils/adminInsights.ts; src/components/details/AdminImpactPanel.tsx</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Unit test and Playwright browser smoke</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>2026-06-24 04:03 UTC</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>investigationSummaryText unit test verifies summary content; Playwright clicked Copy evidence and observed Copied state.</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>No fix needed</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>Clipboard failure is caught so it does not block graph exploration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>TG-094</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Admin investigation</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Saved investigation views</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>As an admin, I want to save a small set of investigation snapshots so I can return to important review contexts during a session.</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Save view stores the current investigation summary in localStorage, caps saved entries at six, displays Saved investigations, and allows individual removal without affecting graph data.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>src/components/details/AdminImpactPanel.tsx; src/styles/05-details.css</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Playwright browser smoke</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2026-06-24 04:03 UTC</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Playwright sample mode cleared localStorage, clicked Save view, confirmed Saved investigations appears and localStorage contains one saved investigation subject.</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>No fix needed</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>Saved views are local browser shortcuts, not tenant-shared records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>TG-095</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Mobile usability</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Responsive workspace and touch navigation</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>As a mobile reviewer, I want the graph, results, filters, and access context reachable without layout overlap so I can inspect a sample tenant from a phone.</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>At &lt;=980px the shell uses natural toolbar height, shows a sticky four-button workspace nav, keeps the graph first, caps the relationship inspector, stacks dense filters, and clamps tutorial highlights inside the viewport.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>src/components/layout/AppShell.tsx; src/components/layout/Toolbar.tsx; src/styles/03-toolbar.css; src/styles/07-responsive.css; src/components/demo/SampleTenantGuide.tsx</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Browser smoke and static verification</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>2026-06-24 04:39 UTC</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Mobile smoke passed at 320px, 390px, and 430px with no horizontal overflow; Results jump lands below sticky nav; desktop 1440px keeps original toolbar and hides mobile nav.</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>No fix needed</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>No separate npm typecheck script exists; direct npx tsc -b and npm run build both passed.</t>
         </is>
       </c>
     </row>
@@ -6480,16 +6587,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="42" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
-    <col min="6" max="6" width="42" customWidth="1"/>
-    <col min="7" max="7" width="42" customWidth="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7490,11 +7601,6 @@
           <t>0 browser console errors; one known Three.js/Vanta warning; no new UX/logistical errors found.</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Verified sample entry/direct route/exit, guide step 3 scroll, real sample apps, CA blocked projection filter, reset-to-sample-user, background/canvas render, selected-anchor no cone/cylinder spotlight, and icon rendering evidence.</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7532,9 +7638,115 @@
           <t>All eight tutorial targets were visible after their guide step activated; zero browser console errors.</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Every targeted sample guide step declares scrollBlock=center; browser confirmed graph canvas, toolbar search, object types, relationships, details, path finder, sign-ins, and Guide button scroll/visibility.</t>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TR-029</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-06-24 04:03 UTC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>TG-077..TG-094 admin impact and sample expansion</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>npx tsc -b --pretty false; npm run lint; npm run test; npm run build; npm audit --audit-level=high; Playwright sample route smoke; vercel --yes; vercel curl /?sampleTenant=1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>68 tests passed; lint/typecheck/build/audit passed; Playwright confirmed 81 objects / 37 relationships, Impact analyzer, broad-target review signals, Copy evidence, and Save view; Vercel preview returned app HTML.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Vite still reports the existing large chunk warning. Dev browser still reports the known duplicate Three.js warning from Vanta plus app Three.js in local development; no app console errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TR-030</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-06-24 04:39 UTC</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TG-095 mobile optimization</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>npm run lint; npx tsc -b; npm run test; npm run build; Playwright browser smoke at 320, 390, 430, and 1440 widths</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Lint passed; TypeScript compiled; 68 tests passed; production build passed; browser smoke found no toolbar/workspace overlap or horizontal overflow after tutorial overlay clamp.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Build still reports the existing large chunk warning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TR-031</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-06-24 04:52 UTC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Thermo-nuclear QA loop and React Doctor remediation</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>npm run lint; npx react-doctor@latest --verbose --scope changed; npm run doctor -- --verbose; npx tsc -b; npm run test; npm run build; git diff --check</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>React Doctor improved from 91/100 with two js-hoist-intl warnings to 100/100 with no issues; lint/typecheck/tests/build passed; strict review fixes applied to admin-impact graph scoping and copy-evidence timer lifecycle.</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Build still reports the existing Vite large-chunk warning; not a lint, React Doctor, or thermo-review blocker.</t>
         </is>
       </c>
     </row>
@@ -7544,20 +7756,24 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="42" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
-    <col min="6" max="6" width="42" customWidth="1"/>
-    <col min="7" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="22" customWidth="1"/>
-    <col min="10" max="10" width="42" customWidth="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7973,11 +8189,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8012,7 +8232,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-23 17:42 UTC</t>
+          <t>2026-06-24 04:39 UTC</t>
         </is>
       </c>
     </row>
@@ -8024,7 +8244,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-23 18:09 UTC</t>
+          <t>2026-06-24 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -8048,7 +8268,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>95</t>
         </is>
       </c>
     </row>
@@ -8060,7 +8280,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tutorial target scrolling retested; all tracked feature stories remain verified with no pending fixes.</t>
+          <t>Thermo-nuclear QA loop, lint, and React Doctor are verified clean; mobile, admin impact, and sample tenant work remain verified.</t>
         </is>
       </c>
     </row>

</xml_diff>